<commit_message>
Update catalog and workbook to approved SunChe prices excluding VAT
</commit_message>
<xml_diff>
--- a/downloads/SunChe_Price_RRP.xlsx
+++ b/downloads/SunChe_Price_RRP.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Зміст" sheetId="1" r:id="R1e83e7e63a9c4f5f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Сонячні панелі" sheetId="2" r:id="Ra35b3d6125b24b4a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FOX ESS" sheetId="3" r:id="R734acee5b4d14947"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="GoodWe" sheetId="4" r:id="R3ba2cd75348d438a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Комплектуючі" sheetId="5" r:id="R9f0cbd6315a24365"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Зміст" sheetId="1" r:id="Rf63afe43207549b9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Сонячні панелі" sheetId="2" r:id="R507373cbb437490f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FOX ESS" sheetId="3" r:id="R72309c1237814de7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="GoodWe" sheetId="4" r:id="Rab09b0553e8c48d3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Комплектуючі" sheetId="5" r:id="Rc9d7c0cf93614d3b"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -226,7 +226,7 @@
         <x:color rgb="FF216345"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFE3F2E9"/>
         </x:patternFill>
       </x:fill>
@@ -236,7 +236,7 @@
         <x:color rgb="FF626F7C"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFEEF1F4"/>
         </x:patternFill>
       </x:fill>
@@ -246,7 +246,7 @@
         <x:color rgb="FF946617"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFF0D3"/>
         </x:patternFill>
       </x:fill>
@@ -256,7 +256,7 @@
         <x:color rgb="FF216345"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFE3F2E9"/>
         </x:patternFill>
       </x:fill>
@@ -266,7 +266,7 @@
         <x:color rgb="FF626F7C"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFEEF1F4"/>
         </x:patternFill>
       </x:fill>
@@ -276,7 +276,7 @@
         <x:color rgb="FF946617"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFF0D3"/>
         </x:patternFill>
       </x:fill>
@@ -286,7 +286,7 @@
         <x:color rgb="FF216345"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFE3F2E9"/>
         </x:patternFill>
       </x:fill>
@@ -296,7 +296,7 @@
         <x:color rgb="FF626F7C"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFEEF1F4"/>
         </x:patternFill>
       </x:fill>
@@ -306,7 +306,7 @@
         <x:color rgb="FF946617"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFF0D3"/>
         </x:patternFill>
       </x:fill>
@@ -316,7 +316,7 @@
         <x:color rgb="FF216345"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFE3F2E9"/>
         </x:patternFill>
       </x:fill>
@@ -326,7 +326,7 @@
         <x:color rgb="FF626F7C"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFEEF1F4"/>
         </x:patternFill>
       </x:fill>
@@ -336,7 +336,7 @@
         <x:color rgb="FF946617"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFF0D3"/>
         </x:patternFill>
       </x:fill>
@@ -357,13 +357,13 @@
     <xdr:ext cx="3960295" cy="2228850"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="1" name="92d8aa90-7edd-40ec-a851-85fdbe54fcb1"/>
+        <xdr:cNvPr id="1" name="/xl/media/image.jpg"/>
         <xdr:cNvPicPr>
           <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R80bb6be512d549d3"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R89f1f12f33b34884"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -389,13 +389,13 @@
     <xdr:ext cx="6348106" cy="914400"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="1" name="6e5f49f8-6eba-49ee-98dc-a775b65eab9d"/>
+        <xdr:cNvPr id="1" name="/xl/media/image2.jpg"/>
         <xdr:cNvPicPr>
           <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Rcf597c7cf9354e5e"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R632a50a126314066"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -421,13 +421,13 @@
     <xdr:ext cx="933450" cy="864057"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="1" name="7ea095d4-1f05-441c-8405-0a651fca4af3"/>
+        <xdr:cNvPr id="1" name="/xl/media/image.png"/>
         <xdr:cNvPicPr>
           <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R5eb0b4b6074248c1"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R9484dec7bba545d1"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -448,13 +448,13 @@
     <xdr:ext cx="5556947" cy="914400"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="2" name="831be25f-34ef-411d-b9ec-7e4047962c43"/>
+        <xdr:cNvPr id="2" name="/xl/media/image3.jpg"/>
         <xdr:cNvPicPr>
           <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Rcb59a44dea3d45f8"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R62d4e482b1aa4d97"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -475,13 +475,13 @@
     <xdr:ext cx="933450" cy="1227831"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="3" name="2d59bd74-b39e-46be-ae6e-9c10348a31cf"/>
+        <xdr:cNvPr id="3" name="/xl/media/image2.png"/>
         <xdr:cNvPicPr>
           <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Rd3c5676c2f38470e"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R73289dc7d7084d88"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -502,13 +502,13 @@
     <xdr:ext cx="933450" cy="1453617"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="4" name="531d9fb3-33d8-4ca0-99a1-f7dfa363f90a"/>
+        <xdr:cNvPr id="4" name="/xl/media/image3.png"/>
         <xdr:cNvPicPr>
           <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R8f29576e01f04c42"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R800e4314420845e6"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -529,13 +529,13 @@
     <xdr:ext cx="933450" cy="1320673"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="5" name="d334e6ae-1844-44da-a61e-748e8088f891"/>
+        <xdr:cNvPr id="5" name="/xl/media/image4.png"/>
         <xdr:cNvPicPr>
           <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R53f438b7b7484f85"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R3d66103933264d50"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -556,13 +556,13 @@
     <xdr:ext cx="933450" cy="961928"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="6" name="f6c15da6-332e-428a-9e0c-4d01de69746f"/>
+        <xdr:cNvPr id="6" name="/xl/media/image5.png"/>
         <xdr:cNvPicPr>
           <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R6307e7771d074fb3"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R5b4b42f3bb0544d8"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -583,13 +583,13 @@
     <xdr:ext cx="933450" cy="1520577"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="7" name="fd33313d-b145-4dfe-96d3-2671b8ced561"/>
+        <xdr:cNvPr id="7" name="/xl/media/image6.png"/>
         <xdr:cNvPicPr>
           <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R26fbbd0cd8494a81"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R552f856284b74cde"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -610,13 +610,13 @@
     <xdr:ext cx="933450" cy="1520577"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="8" name="154582cb-6933-4bdd-a653-4cee9f248cab"/>
+        <xdr:cNvPr id="8" name="/xl/media/image7.png"/>
         <xdr:cNvPicPr>
           <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Rf2fe08688f8744dc"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R28cb27c0d3e142ae"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -637,13 +637,13 @@
     <xdr:ext cx="800100" cy="400050"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="9" name="84026ec9-3685-47d3-bd72-76681e07726a"/>
+        <xdr:cNvPr id="9" name="/xl/media/image8.png"/>
         <xdr:cNvPicPr>
           <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R65e6623e3a334ac3"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Ra6d86a85f83346d8"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -664,13 +664,13 @@
     <xdr:ext cx="933450" cy="602922"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="10" name="fef3b277-ad1c-4fe2-b94d-6210fc97ff5b"/>
+        <xdr:cNvPr id="10" name="/xl/media/image9.png"/>
         <xdr:cNvPicPr>
           <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R87e2e0e380d0497a"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Rdc8c25063030432b"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -691,13 +691,13 @@
     <xdr:ext cx="933450" cy="933450"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="11" name="09cb6a9a-9516-47c7-8529-3b64f4591617"/>
+        <xdr:cNvPr id="11" name="/xl/media/image10.png"/>
         <xdr:cNvPicPr>
           <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Rd3892ae3b96c4512"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R97c50be5cdfb4139"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -718,13 +718,13 @@
     <xdr:ext cx="609600" cy="609600"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="12" name="8b033cb3-f6c1-4718-9c6c-fcbade37ccad"/>
+        <xdr:cNvPr id="12" name="/xl/media/image4.jpg"/>
         <xdr:cNvPicPr>
           <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R8f1184e10ae44b4b"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R7888159aeb9941a1"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -750,13 +750,13 @@
     <xdr:ext cx="707723" cy="952500"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="1" name="15f12cbe-bfb6-411b-ae86-5af295e15901"/>
+        <xdr:cNvPr id="1" name="/xl/media/image11.png"/>
         <xdr:cNvPicPr>
           <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Rb86b03b92c2a4d60"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Rf08c486160a944ce"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -777,13 +777,13 @@
     <xdr:ext cx="933450" cy="1559844"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="2" name="d1cc317d-7c19-4ee2-b43f-d5d7d0df3ab3"/>
+        <xdr:cNvPr id="2" name="/xl/media/image12.png"/>
         <xdr:cNvPicPr>
           <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Rcf61578874554710"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R14434496729443b0"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -804,13 +804,13 @@
     <xdr:ext cx="933450" cy="1004032"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="3" name="0310866a-506d-4486-bdb6-b5a24500f1b8"/>
+        <xdr:cNvPr id="3" name="/xl/media/image13.png"/>
         <xdr:cNvPicPr>
           <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Re2d757a6bd6841de"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Rc146833798134495"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -831,13 +831,13 @@
     <xdr:ext cx="933450" cy="707159"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="4" name="d73ae57c-4ac2-49cc-86c6-44173af4edde"/>
+        <xdr:cNvPr id="4" name="/xl/media/image14.png"/>
         <xdr:cNvPicPr>
           <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R85d50764d1ba4da6"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Rdaaf1530950c4398"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -858,13 +858,13 @@
     <xdr:ext cx="933450" cy="1003168"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="5" name="639b7bb3-57e7-4ae4-b179-3e1da3dce8a2"/>
+        <xdr:cNvPr id="5" name="/xl/media/image15.png"/>
         <xdr:cNvPicPr>
           <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Reb42779eaa374c93"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R5aef02b8d67e4249"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -885,13 +885,13 @@
     <xdr:ext cx="4941138" cy="914400"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="6" name="26936b6f-9193-482e-973a-dfa41e5e9c07"/>
+        <xdr:cNvPr id="6" name="/xl/media/image5.jpg"/>
         <xdr:cNvPicPr>
           <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Rba57391f43224be8"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R289865eb71034519"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -912,13 +912,13 @@
     <xdr:ext cx="933450" cy="929671"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="7" name="8aed298e-be32-47be-a18a-cff6192557f5"/>
+        <xdr:cNvPr id="7" name="/xl/media/image16.png"/>
         <xdr:cNvPicPr>
           <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Rc0c45f976a12498c"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R8da86c34adad41e3"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -939,13 +939,13 @@
     <xdr:ext cx="933450" cy="768646"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="8" name="64fd6ac9-6b64-4066-9763-57bd5a1c7523"/>
+        <xdr:cNvPr id="8" name="/xl/media/image17.png"/>
         <xdr:cNvPicPr>
           <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Rb77bb7ad0d704012"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R9a813524a74a417e"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -966,13 +966,13 @@
     <xdr:ext cx="933450" cy="812505"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="9" name="30d093b4-fa4b-4393-a34f-5e05ea7c1416"/>
+        <xdr:cNvPr id="9" name="/xl/media/image18.png"/>
         <xdr:cNvPicPr>
           <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Rc05de2d59c324c68"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Rd9076eb2f8934a35"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -993,13 +993,13 @@
     <xdr:ext cx="933450" cy="835272"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="10" name="afca383e-8a4a-47c8-9a2f-5fa7d8449d12"/>
+        <xdr:cNvPr id="10" name="/xl/media/image19.png"/>
         <xdr:cNvPicPr>
           <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R8ec3c58c96624fc9"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R399e6db9adc8407d"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -1020,13 +1020,13 @@
     <xdr:ext cx="933450" cy="1116236"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="11" name="aa3e75f8-8756-41d6-8a2b-2ef0c3737bc3"/>
+        <xdr:cNvPr id="11" name="/xl/media/image20.png"/>
         <xdr:cNvPicPr>
           <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R252aa265c0cf483a"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Ra4b7faad0c884b66"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -1047,13 +1047,13 @@
     <xdr:ext cx="933450" cy="1009610"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="12" name="1e9b363c-4ffe-443f-8f7a-2a5a21152c7b"/>
+        <xdr:cNvPr id="12" name="/xl/media/image21.png"/>
         <xdr:cNvPicPr>
           <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R084b23eb5405494b"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R8e150fd3a8444cf6"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -1074,13 +1074,13 @@
     <xdr:ext cx="933450" cy="649835"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="13" name="6c0e0ed0-b85e-402e-bc15-9022633f9daa"/>
+        <xdr:cNvPr id="13" name="/xl/media/image22.png"/>
         <xdr:cNvPicPr>
           <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Rbc8a3c56302d4892"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R86ce3bd2ba2d4a44"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -1101,13 +1101,13 @@
     <xdr:ext cx="933450" cy="743115"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="14" name="fc81de7b-5cfc-47cc-bf43-e384d0026a63"/>
+        <xdr:cNvPr id="14" name="/xl/media/image23.png"/>
         <xdr:cNvPicPr>
           <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R9fd64166908a4e5e"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Ref906a03f6fb45fa"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -1128,13 +1128,13 @@
     <xdr:ext cx="687518" cy="400050"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="15" name="cd1ecb2b-728c-4307-acb2-5c52b79b935b"/>
+        <xdr:cNvPr id="15" name="/xl/media/image24.png"/>
         <xdr:cNvPicPr>
           <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R61cbe42be2d84169"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R282a0722e5604c9b"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -1155,13 +1155,13 @@
     <xdr:ext cx="689719" cy="914400"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="16" name="00878379-f054-4e86-840f-0f71cf5d28fa"/>
+        <xdr:cNvPr id="16" name="/xl/media/image25.png"/>
         <xdr:cNvPicPr>
           <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R02513ddc8f0a4cb4"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R7e5e988e3cdf4023"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -1187,13 +1187,13 @@
     <xdr:ext cx="933450" cy="839286"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="1" name="105ceffc-045a-48e7-905f-03409e77cf61"/>
+        <xdr:cNvPr id="1" name="/xl/media/image26.png"/>
         <xdr:cNvPicPr>
           <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Rd648b94f72684acd"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R88947edb2e6e4d4f"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -1214,13 +1214,13 @@
     <xdr:ext cx="2741861" cy="914400"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="2" name="5c6968fe-572c-4190-b607-448731f3032e"/>
+        <xdr:cNvPr id="2" name="/xl/media/image6.jpg"/>
         <xdr:cNvPicPr>
           <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R6c64f39b541a4dd6"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Rd411136df4604480"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -1241,13 +1241,13 @@
     <xdr:ext cx="933450" cy="933450"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="3" name="fadb8bdf-8c73-4ab2-a7fa-223db6e3e625"/>
+        <xdr:cNvPr id="3" name="/xl/media/image27.png"/>
         <xdr:cNvPicPr>
           <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R8b27b952c826458c"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Ra09507bfdef34222"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -1470,7 +1470,7 @@
     <x:row r="2" ht="48" customHeight="1">
       <x:c r="A2" s="6"/>
       <x:c r="B2" s="6" t="str">
-        <x:v>ПРАЙС / РЕКОМЕНДОВАНІ РОЗДРІБНІ ЦІНИ</x:v>
+        <x:v>ПРАЙС SUNCHE</x:v>
       </x:c>
     </x:row>
     <x:row r="3" ht="48" customHeight="1">
@@ -1515,10 +1515,10 @@
     </x:row>
     <x:row r="8" ht="28.5" customHeight="1">
       <x:c r="A8" s="11" t="str">
-        <x:v>РРЦ</x:v>
+        <x:v>Ціни</x:v>
       </x:c>
       <x:c r="B8" s="11" t="str">
-        <x:v>Єдина ціна у прайсі — рекомендована роздрібна.</x:v>
+        <x:v>Ціни SunChe без ПДВ.</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="28.5" customHeight="1">
@@ -1526,7 +1526,7 @@
         <x:v>Дата</x:v>
       </x:c>
       <x:c r="B9" s="11" t="str">
-        <x:v>Джерело: прайс Nota Trade від 19.10.2026. Наявність і ціну уточнюйте перед замовленням.</x:v>
+        <x:v>Оновлено 26.10.2026. Джерело: Nota Trade від 19.10.2026. Наявність уточнюйте.</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="28.5" customHeight="1">
@@ -1534,7 +1534,7 @@
         <x:v>GoodWe</x:v>
       </x:c>
       <x:c r="B10" s="11" t="str">
-        <x:v>РРЦ не вказана у джерелі. Ціна за запитом.</x:v>
+        <x:v>Ціни GoodWe наведено в євро.</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="28.5" customHeight="1">
@@ -1542,7 +1542,7 @@
         <x:v>Валюта</x:v>
       </x:c>
       <x:c r="B11" s="11" t="str">
-        <x:v>Числові РРЦ наведено в доларах США.</x:v>
+        <x:v>GoodWe — EUR; інші розділи — USD.</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="28.5" customHeight="1">
@@ -1558,7 +1558,7 @@
     <x:mergeCell ref="A1:B1"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb68459cb4c9a4fd1"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf619771522e940d1"/>
 </x:worksheet>
 </file>
 
@@ -1626,7 +1626,8 @@
         <x:v>Datasheet на модель</x:v>
       </x:c>
       <x:c r="J2" s="14" t="str">
-        <x:v>РРЦ, $ / од.</x:v>
+        <x:v>Ціна SunChe, $
+без ПДВ</x:v>
       </x:c>
     </x:row>
     <x:row r="3" ht="0.07500000298023224" customHeight="1">
@@ -1659,7 +1660,7 @@
         <x:v>Datasheet</x:v>
       </x:c>
       <x:c r="J3" s="18" t="n">
-        <x:v>102.52799999999999</x:v>
+        <x:v>78.32</x:v>
       </x:c>
     </x:row>
     <x:row r="4" ht="0.07500000298023224" customHeight="1">
@@ -1692,7 +1693,7 @@
         <x:v>Datasheet</x:v>
       </x:c>
       <x:c r="J4" s="18" t="n">
-        <x:v>106.94999999999999</x:v>
+        <x:v>85.25</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="0.07500000298023224" customHeight="1">
@@ -1723,7 +1724,7 @@
         <x:v>Datasheet</x:v>
       </x:c>
       <x:c r="J5" s="18" t="n">
-        <x:v>0</x:v>
+        <x:v>113.16</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="0.07500000298023224" customHeight="1">
@@ -1756,7 +1757,7 @@
         <x:v>Datasheet</x:v>
       </x:c>
       <x:c r="J6" s="18" t="n">
-        <x:v>100.2456</x:v>
+        <x:v>76.58</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="0.07500000298023224" customHeight="1">
@@ -1789,7 +1790,7 @@
         <x:v>Datasheet</x:v>
       </x:c>
       <x:c r="J7" s="18" t="n">
-        <x:v>129.73379999999997</x:v>
+        <x:v>93.59</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="43.5" customHeight="1">
@@ -1822,7 +1823,7 @@
         <x:v>Datasheet</x:v>
       </x:c>
       <x:c r="J8" s="18" t="n">
-        <x:v>141.31199999999998</x:v>
+        <x:v>109.82</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="0.07500000298023224" customHeight="1">
@@ -1855,7 +1856,7 @@
         <x:v>Datasheet</x:v>
       </x:c>
       <x:c r="J9" s="18" t="n">
-        <x:v>162.80549999999997</x:v>
+        <x:v>118.76</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="0.07500000298023224" customHeight="1">
@@ -1888,7 +1889,7 @@
         <x:v>Datasheet</x:v>
       </x:c>
       <x:c r="J10" s="18" t="n">
-        <x:v>93.96</x:v>
+        <x:v>71.78</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="43.5" customHeight="1">
@@ -1921,7 +1922,7 @@
         <x:v>Datasheet</x:v>
       </x:c>
       <x:c r="J11" s="18" t="n">
-        <x:v>134.688</x:v>
+        <x:v>108.24</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="43.5" customHeight="1">
@@ -1954,7 +1955,7 @@
         <x:v>Datasheet</x:v>
       </x:c>
       <x:c r="J12" s="18" t="n">
-        <x:v>121.14</x:v>
+        <x:v>85.42</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="0.07500000298023224" customHeight="1">
@@ -1987,7 +1988,7 @@
         <x:v>Datasheet</x:v>
       </x:c>
       <x:c r="J13" s="18" t="n">
-        <x:v>135.792</x:v>
+        <x:v>108.24</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="43.5" customHeight="1">
@@ -2020,7 +2021,7 @@
         <x:v>Datasheet</x:v>
       </x:c>
       <x:c r="J14" s="18" t="n">
-        <x:v>139.6278</x:v>
+        <x:v>93.95</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="43.5" customHeight="1">
@@ -2053,7 +2054,7 @@
         <x:v>Datasheet</x:v>
       </x:c>
       <x:c r="J15" s="18" t="n">
-        <x:v>127.22399999999999</x:v>
+        <x:v>90.92</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="0.07500000298023224" customHeight="1">
@@ -2086,7 +2087,7 @@
         <x:v>Datasheet</x:v>
       </x:c>
       <x:c r="J16" s="18" t="n">
-        <x:v>89.712</x:v>
+        <x:v>66.08</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="43.5" customHeight="1">
@@ -2119,7 +2120,7 @@
         <x:v>Datasheet</x:v>
       </x:c>
       <x:c r="J17" s="18" t="n">
-        <x:v>165.888</x:v>
+        <x:v>126.72</x:v>
       </x:c>
     </x:row>
     <x:row r="18" ht="43.5" customHeight="1">
@@ -2152,7 +2153,7 @@
         <x:v>Datasheet</x:v>
       </x:c>
       <x:c r="J18" s="18" t="n">
-        <x:v>150.33599999999998</x:v>
+        <x:v>98.89</x:v>
       </x:c>
     </x:row>
     <x:row r="19" ht="43.5" customHeight="1">
@@ -2182,7 +2183,7 @@
       </x:c>
       <x:c r="I19" s="5"/>
       <x:c r="J19" s="18" t="n">
-        <x:v>150.33599999999998</x:v>
+        <x:v>99.69</x:v>
       </x:c>
     </x:row>
     <x:row r="20" ht="43.5" customHeight="1">
@@ -2215,7 +2216,7 @@
         <x:v>Datasheet</x:v>
       </x:c>
       <x:c r="J20" s="18" t="n">
-        <x:v>150.33599999999998</x:v>
+        <x:v>113.25</x:v>
       </x:c>
     </x:row>
     <x:row r="21" ht="43.5" customHeight="1">
@@ -2245,7 +2246,7 @@
       </x:c>
       <x:c r="I21" s="5"/>
       <x:c r="J21" s="18" t="n">
-        <x:v>150.33599999999998</x:v>
+        <x:v>114.04</x:v>
       </x:c>
     </x:row>
     <x:row r="22" ht="43.5" customHeight="1">
@@ -2275,7 +2276,7 @@
       </x:c>
       <x:c r="I22" s="9"/>
       <x:c r="J22" s="18" t="n">
-        <x:v>150.33599999999998</x:v>
+        <x:v>114.84</x:v>
       </x:c>
     </x:row>
     <x:row r="23" ht="43.5" customHeight="1">
@@ -2356,7 +2357,7 @@
     <x:cfRule type="containsText" dxfId="2" priority="3" operator="containsText" text="очікується"/>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3eed064d9c2148df"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re2770c6be42b44bd"/>
 </x:worksheet>
 </file>
 
@@ -2430,7 +2431,8 @@
         <x:v>Datasheet на модель</x:v>
       </x:c>
       <x:c r="L2" s="14" t="str">
-        <x:v>РРЦ, $ / од.</x:v>
+        <x:v>Ціна SunChe, $
+без ПДВ</x:v>
       </x:c>
     </x:row>
     <x:row r="3" ht="25.5" customHeight="1">
@@ -2483,7 +2485,7 @@
         <x:v>Datasheet</x:v>
       </x:c>
       <x:c r="L4" s="18" t="n">
-        <x:v>947.7</x:v>
+        <x:v>643.5</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="43.5" customHeight="1">
@@ -2517,7 +2519,7 @@
       </x:c>
       <x:c r="K5" s="5"/>
       <x:c r="L5" s="18" t="n">
-        <x:v>985.5</x:v>
+        <x:v>671</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="43.5" customHeight="1">
@@ -2554,7 +2556,7 @@
         <x:v>Datasheet</x:v>
       </x:c>
       <x:c r="L6" s="18" t="n">
-        <x:v>1552.5</x:v>
+        <x:v>1056</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="43.5" customHeight="1">
@@ -2588,7 +2590,7 @@
       </x:c>
       <x:c r="K7" s="5"/>
       <x:c r="L7" s="18" t="n">
-        <x:v>1782</x:v>
+        <x:v>1210</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="25.5" customHeight="1">
@@ -2641,7 +2643,7 @@
         <x:v>Datasheet</x:v>
       </x:c>
       <x:c r="L9" s="18" t="n">
-        <x:v>3226.5</x:v>
+        <x:v>2189</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="43.5" customHeight="1">
@@ -2675,7 +2677,7 @@
       </x:c>
       <x:c r="K10" s="9"/>
       <x:c r="L10" s="18" t="n">
-        <x:v>3645</x:v>
+        <x:v>2475</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="43.5" customHeight="1">
@@ -2709,7 +2711,7 @@
       </x:c>
       <x:c r="K11" s="5"/>
       <x:c r="L11" s="18" t="n">
-        <x:v>3969</x:v>
+        <x:v>2695</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="25.5" customHeight="1">
@@ -2762,7 +2764,7 @@
         <x:v>Datasheet</x:v>
       </x:c>
       <x:c r="L13" s="18" t="n">
-        <x:v>2374.92</x:v>
+        <x:v>1612.6</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="43.5" customHeight="1">
@@ -2796,7 +2798,7 @@
       </x:c>
       <x:c r="K14" s="9"/>
       <x:c r="L14" s="18" t="n">
-        <x:v>2438.1</x:v>
+        <x:v>1655.5</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="43.5" customHeight="1">
@@ -2830,7 +2832,7 @@
       </x:c>
       <x:c r="K15" s="5"/>
       <x:c r="L15" s="18" t="n">
-        <x:v>2499.66</x:v>
+        <x:v>1697.3</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="43.5" customHeight="1">
@@ -2864,7 +2866,7 @@
       </x:c>
       <x:c r="K16" s="9"/>
       <x:c r="L16" s="18" t="n">
-        <x:v>2562.84</x:v>
+        <x:v>1740.2</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="43.5" customHeight="1">
@@ -2898,7 +2900,7 @@
       </x:c>
       <x:c r="K17" s="5"/>
       <x:c r="L17" s="18" t="n">
-        <x:v>2592</x:v>
+        <x:v>1760</x:v>
       </x:c>
     </x:row>
     <x:row r="18" ht="43.5" customHeight="1">
@@ -2932,7 +2934,7 @@
       </x:c>
       <x:c r="K18" s="9"/>
       <x:c r="L18" s="18" t="n">
-        <x:v>2835</x:v>
+        <x:v>1925</x:v>
       </x:c>
     </x:row>
     <x:row r="19" ht="43.5" customHeight="1">
@@ -2969,7 +2971,7 @@
         <x:v>Datasheet</x:v>
       </x:c>
       <x:c r="L19" s="18" t="n">
-        <x:v>3064.5</x:v>
+        <x:v>2079</x:v>
       </x:c>
     </x:row>
     <x:row r="20" ht="43.5" customHeight="1">
@@ -3003,7 +3005,7 @@
       </x:c>
       <x:c r="K20" s="9"/>
       <x:c r="L20" s="18" t="n">
-        <x:v>3645</x:v>
+        <x:v>2475</x:v>
       </x:c>
     </x:row>
     <x:row r="21" ht="25.5" customHeight="1">
@@ -3056,7 +3058,7 @@
         <x:v>Datasheet</x:v>
       </x:c>
       <x:c r="L22" s="18" t="n">
-        <x:v>6075</x:v>
+        <x:v>4125</x:v>
       </x:c>
     </x:row>
     <x:row r="23" ht="43.5" customHeight="1">
@@ -3090,7 +3092,7 @@
       </x:c>
       <x:c r="K23" s="5"/>
       <x:c r="L23" s="18" t="n">
-        <x:v>6640.38</x:v>
+        <x:v>4508.9</x:v>
       </x:c>
     </x:row>
     <x:row r="24" ht="43.5" customHeight="1">
@@ -3124,7 +3126,7 @@
       </x:c>
       <x:c r="K24" s="9"/>
       <x:c r="L24" s="18" t="n">
-        <x:v>7377.48</x:v>
+        <x:v>5009.4</x:v>
       </x:c>
     </x:row>
     <x:row r="25" ht="43.5" customHeight="1">
@@ -3158,7 +3160,7 @@
       </x:c>
       <x:c r="K25" s="5"/>
       <x:c r="L25" s="18" t="n">
-        <x:v>8991</x:v>
+        <x:v>6105</x:v>
       </x:c>
     </x:row>
     <x:row r="26" ht="43.5" customHeight="1">
@@ -3192,7 +3194,7 @@
       </x:c>
       <x:c r="K26" s="9"/>
       <x:c r="L26" s="18" t="n">
-        <x:v>10449</x:v>
+        <x:v>7095</x:v>
       </x:c>
     </x:row>
     <x:row r="27" ht="43.5" customHeight="1">
@@ -3226,7 +3228,7 @@
       </x:c>
       <x:c r="K27" s="5"/>
       <x:c r="L27" s="18" t="n">
-        <x:v>11583</x:v>
+        <x:v>7865</x:v>
       </x:c>
     </x:row>
     <x:row r="28" ht="25.5" customHeight="1">
@@ -3279,7 +3281,7 @@
         <x:v>Datasheet</x:v>
       </x:c>
       <x:c r="L29" s="18" t="n">
-        <x:v>2968.68</x:v>
+        <x:v>2093.3</x:v>
       </x:c>
     </x:row>
     <x:row r="30" ht="43.5" customHeight="1">
@@ -3316,7 +3318,7 @@
         <x:v>Datasheet</x:v>
       </x:c>
       <x:c r="L30" s="18" t="n">
-        <x:v>4574.88</x:v>
+        <x:v>3106.4</x:v>
       </x:c>
     </x:row>
     <x:row r="31" ht="43.5" customHeight="1">
@@ -3350,7 +3352,7 @@
       </x:c>
       <x:c r="K31" s="5"/>
       <x:c r="L31" s="18" t="n">
-        <x:v>6228.9</x:v>
+        <x:v>4229.5</x:v>
       </x:c>
     </x:row>
     <x:row r="32" ht="25.5" customHeight="1">
@@ -3402,7 +3404,7 @@
         <x:v>за запитом</x:v>
       </x:c>
       <x:c r="L33" s="18" t="n">
-        <x:v>57645</x:v>
+        <x:v>42273</x:v>
       </x:c>
     </x:row>
     <x:row r="34" ht="43.5" customHeight="1">
@@ -3436,7 +3438,7 @@
       </x:c>
       <x:c r="K34" s="9"/>
       <x:c r="L34" s="18" t="n">
-        <x:v>60750</x:v>
+        <x:v>44550</x:v>
       </x:c>
     </x:row>
     <x:row r="35" ht="43.5" customHeight="1">
@@ -3470,7 +3472,7 @@
       </x:c>
       <x:c r="K35" s="5"/>
       <x:c r="L35" s="18" t="n">
-        <x:v>65814</x:v>
+        <x:v>48263.6</x:v>
       </x:c>
     </x:row>
     <x:row r="36" ht="43.5" customHeight="1">
@@ -3504,7 +3506,7 @@
       </x:c>
       <x:c r="K36" s="9"/>
       <x:c r="L36" s="18" t="n">
-        <x:v>64161</x:v>
+        <x:v>47051.4</x:v>
       </x:c>
     </x:row>
     <x:row r="37" ht="43.5" customHeight="1">
@@ -3538,7 +3540,7 @@
       </x:c>
       <x:c r="K37" s="5"/>
       <x:c r="L37" s="18" t="n">
-        <x:v>60838.5</x:v>
+        <x:v>44614.9</x:v>
       </x:c>
     </x:row>
     <x:row r="38" ht="48" customHeight="1">
@@ -3572,7 +3574,7 @@
       </x:c>
       <x:c r="K38" s="9"/>
       <x:c r="L38" s="18" t="n">
-        <x:v>58597.5</x:v>
+        <x:v>42971.5</x:v>
       </x:c>
     </x:row>
     <x:row r="39" ht="25.5" customHeight="1">
@@ -3624,7 +3626,7 @@
         <x:v>за запитом</x:v>
       </x:c>
       <x:c r="L40" s="18" t="n">
-        <x:v>60750</x:v>
+        <x:v>44550</x:v>
       </x:c>
     </x:row>
     <x:row r="41" ht="48" customHeight="1">
@@ -3658,7 +3660,7 @@
       </x:c>
       <x:c r="K41" s="5"/>
       <x:c r="L41" s="18" t="n">
-        <x:v>58597.5</x:v>
+        <x:v>42971.5</x:v>
       </x:c>
     </x:row>
     <x:row r="42" ht="43.5" customHeight="1">
@@ -3692,7 +3694,7 @@
       </x:c>
       <x:c r="K42" s="9"/>
       <x:c r="L42" s="18" t="n">
-        <x:v>54000</x:v>
+        <x:v>39600</x:v>
       </x:c>
     </x:row>
     <x:row r="43" ht="25.5" customHeight="1">
@@ -3738,7 +3740,7 @@
       </x:c>
       <x:c r="K44" s="9"/>
       <x:c r="L44" s="18" t="n">
-        <x:v>12580.92</x:v>
+        <x:v>8542.6</x:v>
       </x:c>
     </x:row>
     <x:row r="45" ht="43.5" customHeight="1">
@@ -3764,7 +3766,7 @@
       <x:c r="J45" s="5"/>
       <x:c r="K45" s="5"/>
       <x:c r="L45" s="18" t="n">
-        <x:v>615.6</x:v>
+        <x:v>418</x:v>
       </x:c>
     </x:row>
     <x:row r="46" ht="25.5" customHeight="1">
@@ -3817,7 +3819,7 @@
         <x:v>Datasheet</x:v>
       </x:c>
       <x:c r="L47" s="18" t="n">
-        <x:v>1539</x:v>
+        <x:v>1045</x:v>
       </x:c>
     </x:row>
     <x:row r="48" ht="43.5" customHeight="1">
@@ -3851,7 +3853,7 @@
       </x:c>
       <x:c r="K48" s="9"/>
       <x:c r="L48" s="18" t="n">
-        <x:v>1458</x:v>
+        <x:v>990</x:v>
       </x:c>
     </x:row>
     <x:row r="49" ht="43.5" customHeight="1">
@@ -3888,7 +3890,7 @@
         <x:v>Datasheet</x:v>
       </x:c>
       <x:c r="L49" s="18" t="n">
-        <x:v>2862</x:v>
+        <x:v>1936</x:v>
       </x:c>
     </x:row>
     <x:row r="50" ht="43.5" customHeight="1">
@@ -3922,7 +3924,7 @@
       </x:c>
       <x:c r="K50" s="9"/>
       <x:c r="L50" s="18" t="n">
-        <x:v>1768.5</x:v>
+        <x:v>1199</x:v>
       </x:c>
     </x:row>
     <x:row r="51" ht="60" customHeight="1">
@@ -3955,7 +3957,7 @@
       </x:c>
       <x:c r="K51" s="5"/>
       <x:c r="L51" s="18" t="n">
-        <x:v>4617</x:v>
+        <x:v>3135</x:v>
       </x:c>
     </x:row>
     <x:row r="52" ht="43.5" customHeight="1">
@@ -3992,7 +3994,7 @@
         <x:v>Datasheet</x:v>
       </x:c>
       <x:c r="L52" s="18" t="n">
-        <x:v>1415</x:v>
+        <x:v>979</x:v>
       </x:c>
     </x:row>
     <x:row r="53" ht="43.5" customHeight="1">
@@ -4029,7 +4031,7 @@
         <x:v>Datasheet</x:v>
       </x:c>
       <x:c r="L53" s="18" t="n">
-        <x:v>2760</x:v>
+        <x:v>2046</x:v>
       </x:c>
     </x:row>
     <x:row r="54" ht="48" customHeight="1">
@@ -4066,7 +4068,7 @@
         <x:v>Datasheet</x:v>
       </x:c>
       <x:c r="L54" s="18" t="n">
-        <x:v>1415</x:v>
+        <x:v>979</x:v>
       </x:c>
     </x:row>
     <x:row r="55" ht="48" customHeight="1">
@@ -4103,7 +4105,7 @@
         <x:v>Datasheet</x:v>
       </x:c>
       <x:c r="L55" s="18" t="n">
-        <x:v>2760</x:v>
+        <x:v>2046</x:v>
       </x:c>
     </x:row>
     <x:row r="56" ht="60" customHeight="1">
@@ -4136,7 +4138,7 @@
         <x:v>Datasheet</x:v>
       </x:c>
       <x:c r="L56" s="18" t="n">
-        <x:v>156</x:v>
+        <x:v>130.9</x:v>
       </x:c>
     </x:row>
     <x:row r="57" ht="43.5" customHeight="1">
@@ -4242,7 +4244,7 @@
     <x:cfRule type="containsText" dxfId="5" priority="3" operator="containsText" text="очікується"/>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R07065741577a4c9f"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf2e483b8d0ff48e0"/>
 </x:worksheet>
 </file>
 
@@ -4316,7 +4318,8 @@
         <x:v>Datasheet на модель</x:v>
       </x:c>
       <x:c r="L2" s="14" t="str">
-        <x:v>РРЦ</x:v>
+        <x:v>Ціна SunChe, €
+без ПДВ</x:v>
       </x:c>
     </x:row>
     <x:row r="3" ht="25.5" customHeight="1">
@@ -4363,8 +4366,8 @@
       </x:c>
       <x:c r="J4" s="9"/>
       <x:c r="K4" s="9"/>
-      <x:c r="L4" s="29" t="str">
-        <x:v>Ціна за запитом</x:v>
+      <x:c r="L4" s="29" t="n">
+        <x:v>240.9</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="43.5" customHeight="1">
@@ -4395,8 +4398,8 @@
       </x:c>
       <x:c r="J5" s="5"/>
       <x:c r="K5" s="5"/>
-      <x:c r="L5" s="29" t="str">
-        <x:v>Ціна за запитом</x:v>
+      <x:c r="L5" s="29" t="n">
+        <x:v>247.5</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="43.5" customHeight="1">
@@ -4427,8 +4430,8 @@
       </x:c>
       <x:c r="J6" s="9"/>
       <x:c r="K6" s="9"/>
-      <x:c r="L6" s="29" t="str">
-        <x:v>Ціна за запитом</x:v>
+      <x:c r="L6" s="29" t="n">
+        <x:v>256.3</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="43.5" customHeight="1">
@@ -4459,8 +4462,8 @@
       </x:c>
       <x:c r="J7" s="5"/>
       <x:c r="K7" s="5"/>
-      <x:c r="L7" s="29" t="str">
-        <x:v>Ціна за запитом</x:v>
+      <x:c r="L7" s="29" t="n">
+        <x:v>277.2</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="43.5" customHeight="1">
@@ -4491,8 +4494,8 @@
       </x:c>
       <x:c r="J8" s="9"/>
       <x:c r="K8" s="9"/>
-      <x:c r="L8" s="29" t="str">
-        <x:v>Ціна за запитом</x:v>
+      <x:c r="L8" s="29" t="n">
+        <x:v>290.4</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="43.5" customHeight="1">
@@ -4523,8 +4526,8 @@
       </x:c>
       <x:c r="J9" s="5"/>
       <x:c r="K9" s="5"/>
-      <x:c r="L9" s="29" t="str">
-        <x:v>Ціна за запитом</x:v>
+      <x:c r="L9" s="29" t="n">
+        <x:v>389.4</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="43.5" customHeight="1">
@@ -4555,8 +4558,8 @@
       </x:c>
       <x:c r="J10" s="9"/>
       <x:c r="K10" s="9"/>
-      <x:c r="L10" s="29" t="str">
-        <x:v>Ціна за запитом</x:v>
+      <x:c r="L10" s="29" t="n">
+        <x:v>412.5</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="43.5" customHeight="1">
@@ -4587,8 +4590,8 @@
       </x:c>
       <x:c r="J11" s="5"/>
       <x:c r="K11" s="5"/>
-      <x:c r="L11" s="29" t="str">
-        <x:v>Ціна за запитом</x:v>
+      <x:c r="L11" s="29" t="n">
+        <x:v>434.5</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="43.5" customHeight="1">
@@ -4619,8 +4622,8 @@
       </x:c>
       <x:c r="J12" s="9"/>
       <x:c r="K12" s="9"/>
-      <x:c r="L12" s="29" t="str">
-        <x:v>Ціна за запитом</x:v>
+      <x:c r="L12" s="29" t="n">
+        <x:v>456.5</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="43.5" customHeight="1">
@@ -4651,8 +4654,8 @@
       </x:c>
       <x:c r="J13" s="5"/>
       <x:c r="K13" s="5"/>
-      <x:c r="L13" s="29" t="str">
-        <x:v>Ціна за запитом</x:v>
+      <x:c r="L13" s="29" t="n">
+        <x:v>479.6</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="43.5" customHeight="1">
@@ -4683,8 +4686,8 @@
       </x:c>
       <x:c r="J14" s="9"/>
       <x:c r="K14" s="9"/>
-      <x:c r="L14" s="29" t="str">
-        <x:v>Ціна за запитом</x:v>
+      <x:c r="L14" s="29" t="n">
+        <x:v>557.7</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="43.5" customHeight="1">
@@ -4715,8 +4718,8 @@
       </x:c>
       <x:c r="J15" s="5"/>
       <x:c r="K15" s="5"/>
-      <x:c r="L15" s="29" t="str">
-        <x:v>Ціна за запитом</x:v>
+      <x:c r="L15" s="29" t="n">
+        <x:v>594</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="43.5" customHeight="1">
@@ -4747,8 +4750,8 @@
       </x:c>
       <x:c r="J16" s="9"/>
       <x:c r="K16" s="9"/>
-      <x:c r="L16" s="29" t="str">
-        <x:v>Ціна за запитом</x:v>
+      <x:c r="L16" s="29" t="n">
+        <x:v>638</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="25.5" customHeight="1">
@@ -4795,8 +4798,8 @@
       </x:c>
       <x:c r="J18" s="9"/>
       <x:c r="K18" s="9"/>
-      <x:c r="L18" s="29" t="str">
-        <x:v>Ціна за запитом</x:v>
+      <x:c r="L18" s="29" t="n">
+        <x:v>731.05</x:v>
       </x:c>
     </x:row>
     <x:row r="19" ht="43.5" customHeight="1">
@@ -4827,8 +4830,8 @@
       </x:c>
       <x:c r="J19" s="5"/>
       <x:c r="K19" s="5"/>
-      <x:c r="L19" s="29" t="str">
-        <x:v>Ціна за запитом</x:v>
+      <x:c r="L19" s="29" t="n">
+        <x:v>810.94</x:v>
       </x:c>
     </x:row>
     <x:row r="20" ht="43.5" customHeight="1">
@@ -4859,8 +4862,8 @@
       </x:c>
       <x:c r="J20" s="9"/>
       <x:c r="K20" s="9"/>
-      <x:c r="L20" s="29" t="str">
-        <x:v>Ціна за запитом</x:v>
+      <x:c r="L20" s="29" t="n">
+        <x:v>837.73</x:v>
       </x:c>
     </x:row>
     <x:row r="21" ht="25.5" customHeight="1">
@@ -4907,8 +4910,8 @@
       </x:c>
       <x:c r="J22" s="9"/>
       <x:c r="K22" s="9"/>
-      <x:c r="L22" s="29" t="str">
-        <x:v>Ціна за запитом</x:v>
+      <x:c r="L22" s="29" t="n">
+        <x:v>989.69</x:v>
       </x:c>
     </x:row>
     <x:row r="23" ht="43.5" customHeight="1">
@@ -4939,8 +4942,8 @@
       </x:c>
       <x:c r="J23" s="5"/>
       <x:c r="K23" s="5"/>
-      <x:c r="L23" s="29" t="str">
-        <x:v>Ціна за запитом</x:v>
+      <x:c r="L23" s="29" t="n">
+        <x:v>1053.55</x:v>
       </x:c>
     </x:row>
     <x:row r="24" ht="43.5" customHeight="1">
@@ -4971,8 +4974,8 @@
       </x:c>
       <x:c r="J24" s="9"/>
       <x:c r="K24" s="9"/>
-      <x:c r="L24" s="29" t="str">
-        <x:v>Ціна за запитом</x:v>
+      <x:c r="L24" s="29" t="n">
+        <x:v>1167.76</x:v>
       </x:c>
     </x:row>
     <x:row r="25" ht="43.5" customHeight="1">
@@ -5003,8 +5006,8 @@
       </x:c>
       <x:c r="J25" s="5"/>
       <x:c r="K25" s="5"/>
-      <x:c r="L25" s="29" t="str">
-        <x:v>Ціна за запитом</x:v>
+      <x:c r="L25" s="29" t="n">
+        <x:v>1140.7</x:v>
       </x:c>
     </x:row>
     <x:row r="26" ht="43.5" customHeight="1">
@@ -5035,8 +5038,8 @@
       </x:c>
       <x:c r="J26" s="9"/>
       <x:c r="K26" s="9"/>
-      <x:c r="L26" s="29" t="str">
-        <x:v>Ціна за запитом</x:v>
+      <x:c r="L26" s="29" t="n">
+        <x:v>1833.35</x:v>
       </x:c>
     </x:row>
     <x:row r="27" ht="43.5" customHeight="1">
@@ -5067,8 +5070,8 @@
       </x:c>
       <x:c r="J27" s="5"/>
       <x:c r="K27" s="5"/>
-      <x:c r="L27" s="29" t="str">
-        <x:v>Ціна за запитом</x:v>
+      <x:c r="L27" s="29" t="n">
+        <x:v>1906.19</x:v>
       </x:c>
     </x:row>
     <x:row r="28" ht="43.5" customHeight="1">
@@ -5099,8 +5102,8 @@
       </x:c>
       <x:c r="J28" s="9"/>
       <x:c r="K28" s="9"/>
-      <x:c r="L28" s="29" t="str">
-        <x:v>Ціна за запитом</x:v>
+      <x:c r="L28" s="29" t="n">
+        <x:v>1558.7</x:v>
       </x:c>
     </x:row>
     <x:row r="29" ht="43.5" customHeight="1">
@@ -5131,8 +5134,8 @@
       </x:c>
       <x:c r="J29" s="5"/>
       <x:c r="K29" s="5"/>
-      <x:c r="L29" s="29" t="str">
-        <x:v>Ціна за запитом</x:v>
+      <x:c r="L29" s="29" t="n">
+        <x:v>2423.92</x:v>
       </x:c>
     </x:row>
     <x:row r="30" ht="43.5" customHeight="1">
@@ -5163,8 +5166,8 @@
       </x:c>
       <x:c r="J30" s="9"/>
       <x:c r="K30" s="9"/>
-      <x:c r="L30" s="29" t="str">
-        <x:v>Ціна за запитом</x:v>
+      <x:c r="L30" s="29" t="n">
+        <x:v>2826.82</x:v>
       </x:c>
     </x:row>
     <x:row r="31" ht="43.5" customHeight="1">
@@ -5195,8 +5198,8 @@
       </x:c>
       <x:c r="J31" s="5"/>
       <x:c r="K31" s="5"/>
-      <x:c r="L31" s="29" t="str">
-        <x:v>Ціна за запитом</x:v>
+      <x:c r="L31" s="29" t="n">
+        <x:v>2857.83</x:v>
       </x:c>
     </x:row>
     <x:row r="32" ht="43.5" customHeight="1">
@@ -5227,8 +5230,8 @@
       </x:c>
       <x:c r="J32" s="9"/>
       <x:c r="K32" s="9"/>
-      <x:c r="L32" s="29" t="str">
-        <x:v>Ціна за запитом</x:v>
+      <x:c r="L32" s="29" t="n">
+        <x:v>3100.9</x:v>
       </x:c>
     </x:row>
     <x:row r="33" ht="43.5" customHeight="1">
@@ -5261,8 +5264,8 @@
         <x:v>60</x:v>
       </x:c>
       <x:c r="K33" s="5"/>
-      <x:c r="L33" s="29" t="str">
-        <x:v>Ціна за запитом</x:v>
+      <x:c r="L33" s="29" t="n">
+        <x:v>3405.6</x:v>
       </x:c>
     </x:row>
     <x:row r="34" ht="25.5" customHeight="1">
@@ -5309,8 +5312,8 @@
       </x:c>
       <x:c r="J35" s="5"/>
       <x:c r="K35" s="5"/>
-      <x:c r="L35" s="29" t="str">
-        <x:v>Ціна за запитом</x:v>
+      <x:c r="L35" s="29" t="n">
+        <x:v>738.69</x:v>
       </x:c>
     </x:row>
     <x:row r="36" ht="43.5" customHeight="1">
@@ -5341,8 +5344,8 @@
       </x:c>
       <x:c r="J36" s="9"/>
       <x:c r="K36" s="9"/>
-      <x:c r="L36" s="29" t="str">
-        <x:v>Ціна за запитом</x:v>
+      <x:c r="L36" s="29" t="n">
+        <x:v>764.59</x:v>
       </x:c>
     </x:row>
     <x:row r="37" ht="43.5" customHeight="1">
@@ -5373,8 +5376,8 @@
       </x:c>
       <x:c r="J37" s="5"/>
       <x:c r="K37" s="5"/>
-      <x:c r="L37" s="29" t="str">
-        <x:v>Ціна за запитом</x:v>
+      <x:c r="L37" s="29" t="n">
+        <x:v>781</x:v>
       </x:c>
     </x:row>
     <x:row r="38" ht="43.5" customHeight="1">
@@ -5405,8 +5408,8 @@
       </x:c>
       <x:c r="J38" s="9"/>
       <x:c r="K38" s="9"/>
-      <x:c r="L38" s="29" t="str">
-        <x:v>Ціна за запитом</x:v>
+      <x:c r="L38" s="29" t="n">
+        <x:v>1007.91</x:v>
       </x:c>
     </x:row>
     <x:row r="39" ht="43.5" customHeight="1">
@@ -5437,8 +5440,8 @@
       </x:c>
       <x:c r="J39" s="5"/>
       <x:c r="K39" s="5"/>
-      <x:c r="L39" s="29" t="str">
-        <x:v>Ціна за запитом</x:v>
+      <x:c r="L39" s="29" t="n">
+        <x:v>1111.83</x:v>
       </x:c>
     </x:row>
     <x:row r="40" ht="43.5" customHeight="1">
@@ -5469,8 +5472,8 @@
       </x:c>
       <x:c r="J40" s="9"/>
       <x:c r="K40" s="9"/>
-      <x:c r="L40" s="29" t="str">
-        <x:v>Ціна за запитом</x:v>
+      <x:c r="L40" s="29" t="n">
+        <x:v>1210.53</x:v>
       </x:c>
     </x:row>
     <x:row r="41" ht="43.5" customHeight="1">
@@ -5501,8 +5504,8 @@
       </x:c>
       <x:c r="J41" s="5"/>
       <x:c r="K41" s="5"/>
-      <x:c r="L41" s="29" t="str">
-        <x:v>Ціна за запитом</x:v>
+      <x:c r="L41" s="29" t="n">
+        <x:v>781</x:v>
       </x:c>
     </x:row>
     <x:row r="42" ht="43.5" customHeight="1">
@@ -5533,8 +5536,8 @@
       </x:c>
       <x:c r="J42" s="9"/>
       <x:c r="K42" s="9"/>
-      <x:c r="L42" s="29" t="str">
-        <x:v>Ціна за запитом</x:v>
+      <x:c r="L42" s="29" t="n">
+        <x:v>841.16</x:v>
       </x:c>
     </x:row>
     <x:row r="43" ht="43.5" customHeight="1">
@@ -5565,8 +5568,8 @@
       </x:c>
       <x:c r="J43" s="5"/>
       <x:c r="K43" s="5"/>
-      <x:c r="L43" s="29" t="str">
-        <x:v>Ціна за запитом</x:v>
+      <x:c r="L43" s="29" t="n">
+        <x:v>856.28</x:v>
       </x:c>
     </x:row>
     <x:row r="44" ht="43.5" customHeight="1">
@@ -5597,8 +5600,8 @@
       </x:c>
       <x:c r="J44" s="9"/>
       <x:c r="K44" s="9"/>
-      <x:c r="L44" s="29" t="str">
-        <x:v>Ціна за запитом</x:v>
+      <x:c r="L44" s="29" t="n">
+        <x:v>738.1</x:v>
       </x:c>
     </x:row>
     <x:row r="45" ht="43.5" customHeight="1">
@@ -5629,8 +5632,8 @@
       </x:c>
       <x:c r="J45" s="5"/>
       <x:c r="K45" s="5"/>
-      <x:c r="L45" s="29" t="str">
-        <x:v>Ціна за запитом</x:v>
+      <x:c r="L45" s="29" t="n">
+        <x:v>862.4</x:v>
       </x:c>
     </x:row>
     <x:row r="46" ht="43.5" customHeight="1">
@@ -5661,8 +5664,8 @@
       </x:c>
       <x:c r="J46" s="9"/>
       <x:c r="K46" s="9"/>
-      <x:c r="L46" s="29" t="str">
-        <x:v>Ціна за запитом</x:v>
+      <x:c r="L46" s="29" t="n">
+        <x:v>918.5</x:v>
       </x:c>
     </x:row>
     <x:row r="47" ht="25.5" customHeight="1">
@@ -5709,8 +5712,8 @@
       </x:c>
       <x:c r="J48" s="9"/>
       <x:c r="K48" s="9"/>
-      <x:c r="L48" s="29" t="str">
-        <x:v>Ціна за запитом</x:v>
+      <x:c r="L48" s="29" t="n">
+        <x:v>1263.41</x:v>
       </x:c>
     </x:row>
     <x:row r="49" ht="43.5" customHeight="1">
@@ -5741,8 +5744,8 @@
       </x:c>
       <x:c r="J49" s="5"/>
       <x:c r="K49" s="5"/>
-      <x:c r="L49" s="29" t="str">
-        <x:v>Ціна за запитом</x:v>
+      <x:c r="L49" s="29" t="n">
+        <x:v>1315.2</x:v>
       </x:c>
     </x:row>
     <x:row r="50" ht="43.5" customHeight="1">
@@ -5773,8 +5776,8 @@
       </x:c>
       <x:c r="J50" s="9"/>
       <x:c r="K50" s="9"/>
-      <x:c r="L50" s="29" t="str">
-        <x:v>Ціна за запитом</x:v>
+      <x:c r="L50" s="29" t="n">
+        <x:v>1372.44</x:v>
       </x:c>
     </x:row>
     <x:row r="51" ht="43.5" customHeight="1">
@@ -5805,8 +5808,8 @@
       </x:c>
       <x:c r="J51" s="5"/>
       <x:c r="K51" s="5"/>
-      <x:c r="L51" s="29" t="str">
-        <x:v>Ціна за запитом</x:v>
+      <x:c r="L51" s="29" t="n">
+        <x:v>1433.77</x:v>
       </x:c>
     </x:row>
     <x:row r="52" ht="25.5" customHeight="1">
@@ -5853,8 +5856,8 @@
       </x:c>
       <x:c r="J53" s="5"/>
       <x:c r="K53" s="5"/>
-      <x:c r="L53" s="29" t="str">
-        <x:v>Ціна за запитом</x:v>
+      <x:c r="L53" s="29" t="n">
+        <x:v>1183.62</x:v>
       </x:c>
     </x:row>
     <x:row r="54" ht="43.5" customHeight="1">
@@ -5885,8 +5888,8 @@
       </x:c>
       <x:c r="J54" s="9"/>
       <x:c r="K54" s="9"/>
-      <x:c r="L54" s="29" t="str">
-        <x:v>Ціна за запитом</x:v>
+      <x:c r="L54" s="29" t="n">
+        <x:v>1211.95</x:v>
       </x:c>
     </x:row>
     <x:row r="55" ht="43.5" customHeight="1">
@@ -5917,8 +5920,8 @@
       </x:c>
       <x:c r="J55" s="5"/>
       <x:c r="K55" s="5"/>
-      <x:c r="L55" s="29" t="str">
-        <x:v>Ціна за запитом</x:v>
+      <x:c r="L55" s="29" t="n">
+        <x:v>1231.27</x:v>
       </x:c>
     </x:row>
     <x:row r="56" ht="43.5" customHeight="1">
@@ -5949,8 +5952,8 @@
       </x:c>
       <x:c r="J56" s="9"/>
       <x:c r="K56" s="9"/>
-      <x:c r="L56" s="29" t="str">
-        <x:v>Ціна за запитом</x:v>
+      <x:c r="L56" s="29" t="n">
+        <x:v>1268.62</x:v>
       </x:c>
     </x:row>
     <x:row r="57" ht="43.5" customHeight="1">
@@ -5981,8 +5984,8 @@
       </x:c>
       <x:c r="J57" s="5"/>
       <x:c r="K57" s="5"/>
-      <x:c r="L57" s="29" t="str">
-        <x:v>Ціна за запитом</x:v>
+      <x:c r="L57" s="29" t="n">
+        <x:v>1298.24</x:v>
       </x:c>
     </x:row>
     <x:row r="58" ht="25.5" customHeight="1">
@@ -6029,8 +6032,8 @@
       </x:c>
       <x:c r="J59" s="5"/>
       <x:c r="K59" s="5"/>
-      <x:c r="L59" s="29" t="str">
-        <x:v>Ціна за запитом</x:v>
+      <x:c r="L59" s="29" t="n">
+        <x:v>2047.21</x:v>
       </x:c>
     </x:row>
     <x:row r="60" ht="43.5" customHeight="1">
@@ -6061,8 +6064,8 @@
       </x:c>
       <x:c r="J60" s="9"/>
       <x:c r="K60" s="9"/>
-      <x:c r="L60" s="29" t="str">
-        <x:v>Ціна за запитом</x:v>
+      <x:c r="L60" s="29" t="n">
+        <x:v>2144.11</x:v>
       </x:c>
     </x:row>
     <x:row r="61" ht="43.5" customHeight="1">
@@ -6093,8 +6096,8 @@
       </x:c>
       <x:c r="J61" s="5"/>
       <x:c r="K61" s="5"/>
-      <x:c r="L61" s="29" t="str">
-        <x:v>Ціна за запитом</x:v>
+      <x:c r="L61" s="29" t="n">
+        <x:v>2323.2</x:v>
       </x:c>
     </x:row>
     <x:row r="62" ht="43.5" customHeight="1">
@@ -6125,8 +6128,8 @@
       </x:c>
       <x:c r="J62" s="9"/>
       <x:c r="K62" s="9"/>
-      <x:c r="L62" s="29" t="str">
-        <x:v>Ціна за запитом</x:v>
+      <x:c r="L62" s="29" t="n">
+        <x:v>2471.62</x:v>
       </x:c>
     </x:row>
     <x:row r="63" ht="43.5" customHeight="1">
@@ -6157,8 +6160,8 @@
       </x:c>
       <x:c r="J63" s="5"/>
       <x:c r="K63" s="5"/>
-      <x:c r="L63" s="29" t="str">
-        <x:v>Ціна за запитом</x:v>
+      <x:c r="L63" s="29" t="n">
+        <x:v>2785.2</x:v>
       </x:c>
     </x:row>
     <x:row r="64" ht="43.5" customHeight="1">
@@ -6189,8 +6192,8 @@
       </x:c>
       <x:c r="J64" s="9"/>
       <x:c r="K64" s="9"/>
-      <x:c r="L64" s="29" t="str">
-        <x:v>Ціна за запитом</x:v>
+      <x:c r="L64" s="29" t="n">
+        <x:v>2982.1</x:v>
       </x:c>
     </x:row>
     <x:row r="65" ht="43.5" customHeight="1">
@@ -6221,8 +6224,8 @@
       </x:c>
       <x:c r="J65" s="5"/>
       <x:c r="K65" s="5"/>
-      <x:c r="L65" s="29" t="str">
-        <x:v>Ціна за запитом</x:v>
+      <x:c r="L65" s="29" t="n">
+        <x:v>3770.8</x:v>
       </x:c>
     </x:row>
     <x:row r="66" ht="43.5" customHeight="1">
@@ -6255,8 +6258,8 @@
         <x:v>60</x:v>
       </x:c>
       <x:c r="K66" s="9"/>
-      <x:c r="L66" s="29" t="str">
-        <x:v>Ціна за запитом</x:v>
+      <x:c r="L66" s="29" t="n">
+        <x:v>3889.6</x:v>
       </x:c>
     </x:row>
     <x:row r="67" ht="25.5" customHeight="1">
@@ -6301,8 +6304,8 @@
       </x:c>
       <x:c r="J68" s="9"/>
       <x:c r="K68" s="9"/>
-      <x:c r="L68" s="29" t="str">
-        <x:v>Ціна за запитом</x:v>
+      <x:c r="L68" s="29" t="n">
+        <x:v>867.06</x:v>
       </x:c>
     </x:row>
     <x:row r="69" ht="43.5" customHeight="1">
@@ -6331,8 +6334,8 @@
       </x:c>
       <x:c r="J69" s="5"/>
       <x:c r="K69" s="5"/>
-      <x:c r="L69" s="29" t="str">
-        <x:v>Ціна за запитом</x:v>
+      <x:c r="L69" s="29" t="n">
+        <x:v>1038.9</x:v>
       </x:c>
     </x:row>
     <x:row r="70" ht="25.5" customHeight="1">
@@ -6375,8 +6378,8 @@
       </x:c>
       <x:c r="J71" s="5"/>
       <x:c r="K71" s="5"/>
-      <x:c r="L71" s="29" t="str">
-        <x:v>Ціна за запитом</x:v>
+      <x:c r="L71" s="29" t="n">
+        <x:v>1295.32</x:v>
       </x:c>
     </x:row>
     <x:row r="72" ht="25.5" customHeight="1">
@@ -6419,8 +6422,8 @@
       </x:c>
       <x:c r="J73" s="5"/>
       <x:c r="K73" s="5"/>
-      <x:c r="L73" s="29" t="str">
-        <x:v>Ціна за запитом</x:v>
+      <x:c r="L73" s="29" t="n">
+        <x:v>1563.82</x:v>
       </x:c>
     </x:row>
     <x:row r="74" ht="43.5" customHeight="1">
@@ -6447,8 +6450,8 @@
       </x:c>
       <x:c r="J74" s="9"/>
       <x:c r="K74" s="9"/>
-      <x:c r="L74" s="29" t="str">
-        <x:v>Ціна за запитом</x:v>
+      <x:c r="L74" s="29" t="n">
+        <x:v>3447.39</x:v>
       </x:c>
     </x:row>
     <x:row r="75" ht="43.5" customHeight="1">
@@ -6475,8 +6478,8 @@
       </x:c>
       <x:c r="J75" s="5"/>
       <x:c r="K75" s="5"/>
-      <x:c r="L75" s="29" t="str">
-        <x:v>Ціна за запитом</x:v>
+      <x:c r="L75" s="29" t="n">
+        <x:v>3462.37</x:v>
       </x:c>
     </x:row>
     <x:row r="76" ht="43.5" customHeight="1">
@@ -6503,8 +6506,8 @@
       </x:c>
       <x:c r="J76" s="9"/>
       <x:c r="K76" s="9"/>
-      <x:c r="L76" s="29" t="str">
-        <x:v>Ціна за запитом</x:v>
+      <x:c r="L76" s="29" t="n">
+        <x:v>3636</x:v>
       </x:c>
     </x:row>
     <x:row r="77" ht="43.5" customHeight="1">
@@ -6531,8 +6534,8 @@
       </x:c>
       <x:c r="J77" s="5"/>
       <x:c r="K77" s="5"/>
-      <x:c r="L77" s="29" t="str">
-        <x:v>Ціна за запитом</x:v>
+      <x:c r="L77" s="29" t="n">
+        <x:v>3654.73</x:v>
       </x:c>
     </x:row>
     <x:row r="78" ht="43.5" customHeight="1">
@@ -6559,8 +6562,8 @@
       </x:c>
       <x:c r="J78" s="9"/>
       <x:c r="K78" s="9"/>
-      <x:c r="L78" s="29" t="str">
-        <x:v>Ціна за запитом</x:v>
+      <x:c r="L78" s="29" t="n">
+        <x:v>16663.76</x:v>
       </x:c>
     </x:row>
     <x:row r="79" ht="43.5" customHeight="1">
@@ -6587,8 +6590,8 @@
       </x:c>
       <x:c r="J79" s="5"/>
       <x:c r="K79" s="5"/>
-      <x:c r="L79" s="29" t="str">
-        <x:v>Ціна за запитом</x:v>
+      <x:c r="L79" s="29" t="n">
+        <x:v>15846.31</x:v>
       </x:c>
     </x:row>
     <x:row r="80" ht="43.5" customHeight="1">
@@ -6615,8 +6618,8 @@
       </x:c>
       <x:c r="J80" s="9"/>
       <x:c r="K80" s="9"/>
-      <x:c r="L80" s="29" t="str">
-        <x:v>Ціна за запитом</x:v>
+      <x:c r="L80" s="29" t="n">
+        <x:v>19030</x:v>
       </x:c>
     </x:row>
     <x:row r="81" ht="43.5" customHeight="1">
@@ -6645,8 +6648,8 @@
         <x:v>60</x:v>
       </x:c>
       <x:c r="K81" s="5"/>
-      <x:c r="L81" s="29" t="str">
-        <x:v>Ціна за запитом</x:v>
+      <x:c r="L81" s="29" t="n">
+        <x:v>20341.2</x:v>
       </x:c>
     </x:row>
     <x:row r="82" ht="25.5" customHeight="1">
@@ -6690,8 +6693,8 @@
         <x:f>IFERROR(HYPERLINK("https://drive.google.com/file/d/1es0RpKLsh89dUDHIClbvqlMHx4mfb42O/view?usp=drive_link","Datasheet"),"Datasheet")</x:f>
         <x:v>Datasheet</x:v>
       </x:c>
-      <x:c r="L83" s="29" t="str">
-        <x:v>Ціна за запитом</x:v>
+      <x:c r="L83" s="29" t="n">
+        <x:v>42137.7</x:v>
       </x:c>
     </x:row>
     <x:row r="84" ht="25.5" customHeight="1">
@@ -6736,8 +6739,8 @@
       </x:c>
       <x:c r="J85" s="5"/>
       <x:c r="K85" s="5"/>
-      <x:c r="L85" s="29" t="str">
-        <x:v>Ціна за запитом</x:v>
+      <x:c r="L85" s="29" t="n">
+        <x:v>57.2</x:v>
       </x:c>
     </x:row>
     <x:row r="86" ht="43.5" customHeight="1">
@@ -6766,8 +6769,8 @@
       </x:c>
       <x:c r="J86" s="9"/>
       <x:c r="K86" s="9"/>
-      <x:c r="L86" s="29" t="str">
-        <x:v>Ціна за запитом</x:v>
+      <x:c r="L86" s="29" t="n">
+        <x:v>60.5</x:v>
       </x:c>
     </x:row>
     <x:row r="87" ht="43.5" customHeight="1">
@@ -6796,8 +6799,8 @@
       </x:c>
       <x:c r="J87" s="5"/>
       <x:c r="K87" s="5"/>
-      <x:c r="L87" s="29" t="str">
-        <x:v>Ціна за запитом</x:v>
+      <x:c r="L87" s="29" t="n">
+        <x:v>133.1</x:v>
       </x:c>
     </x:row>
     <x:row r="88" ht="43.5" customHeight="1">
@@ -6828,8 +6831,8 @@
         <x:v>60</x:v>
       </x:c>
       <x:c r="K88" s="9"/>
-      <x:c r="L88" s="29" t="str">
-        <x:v>Ціна за запитом</x:v>
+      <x:c r="L88" s="29" t="n">
+        <x:v>93.94</x:v>
       </x:c>
     </x:row>
     <x:row r="89" ht="43.5" customHeight="1">
@@ -6858,8 +6861,8 @@
       </x:c>
       <x:c r="J89" s="5"/>
       <x:c r="K89" s="5"/>
-      <x:c r="L89" s="29" t="str">
-        <x:v>Ціна за запитом</x:v>
+      <x:c r="L89" s="29" t="n">
+        <x:v>307.62</x:v>
       </x:c>
     </x:row>
     <x:row r="90" ht="43.5" customHeight="1">
@@ -6888,8 +6891,8 @@
       </x:c>
       <x:c r="J90" s="9"/>
       <x:c r="K90" s="9"/>
-      <x:c r="L90" s="29" t="str">
-        <x:v>Ціна за запитом</x:v>
+      <x:c r="L90" s="29" t="n">
+        <x:v>307.62</x:v>
       </x:c>
     </x:row>
     <x:row r="91" ht="43.5" customHeight="1">
@@ -6918,8 +6921,8 @@
       </x:c>
       <x:c r="J91" s="5"/>
       <x:c r="K91" s="5"/>
-      <x:c r="L91" s="29" t="str">
-        <x:v>Ціна за запитом</x:v>
+      <x:c r="L91" s="29" t="n">
+        <x:v>201.63</x:v>
       </x:c>
     </x:row>
     <x:row r="92" ht="43.5" customHeight="1">
@@ -6948,8 +6951,8 @@
       </x:c>
       <x:c r="J92" s="9"/>
       <x:c r="K92" s="9"/>
-      <x:c r="L92" s="29" t="str">
-        <x:v>Ціна за запитом</x:v>
+      <x:c r="L92" s="29" t="n">
+        <x:v>417.48</x:v>
       </x:c>
     </x:row>
     <x:row r="93" ht="43.5" customHeight="1">
@@ -6978,8 +6981,8 @@
       </x:c>
       <x:c r="J93" s="5"/>
       <x:c r="K93" s="5"/>
-      <x:c r="L93" s="29" t="str">
-        <x:v>Ціна за запитом</x:v>
+      <x:c r="L93" s="29" t="n">
+        <x:v>429</x:v>
       </x:c>
     </x:row>
     <x:row r="94" ht="43.5" customHeight="1">
@@ -7008,8 +7011,8 @@
       </x:c>
       <x:c r="J94" s="9"/>
       <x:c r="K94" s="9"/>
-      <x:c r="L94" s="29" t="str">
-        <x:v>Ціна за запитом</x:v>
+      <x:c r="L94" s="29" t="n">
+        <x:v>804.76</x:v>
       </x:c>
     </x:row>
     <x:row r="95" ht="43.5" customHeight="1">
@@ -7038,8 +7041,8 @@
       </x:c>
       <x:c r="J95" s="5"/>
       <x:c r="K95" s="5"/>
-      <x:c r="L95" s="29" t="str">
-        <x:v>Ціна за запитом</x:v>
+      <x:c r="L95" s="29" t="n">
+        <x:v>1049.51</x:v>
       </x:c>
     </x:row>
     <x:row r="96" ht="43.5" customHeight="1">
@@ -7068,8 +7071,8 @@
       </x:c>
       <x:c r="J96" s="9"/>
       <x:c r="K96" s="9"/>
-      <x:c r="L96" s="29" t="str">
-        <x:v>Ціна за запитом</x:v>
+      <x:c r="L96" s="29" t="n">
+        <x:v>1403.66</x:v>
       </x:c>
     </x:row>
     <x:row r="97" ht="43.5" customHeight="1">
@@ -7098,8 +7101,8 @@
       </x:c>
       <x:c r="J97" s="5"/>
       <x:c r="K97" s="5"/>
-      <x:c r="L97" s="29" t="str">
-        <x:v>Ціна за запитом</x:v>
+      <x:c r="L97" s="29" t="n">
+        <x:v>1213.66</x:v>
       </x:c>
     </x:row>
     <x:row r="98" ht="43.5" customHeight="1">
@@ -7128,8 +7131,8 @@
       </x:c>
       <x:c r="J98" s="9"/>
       <x:c r="K98" s="9"/>
-      <x:c r="L98" s="29" t="str">
-        <x:v>Ціна за запитом</x:v>
+      <x:c r="L98" s="29" t="n">
+        <x:v>1437.26</x:v>
       </x:c>
     </x:row>
     <x:row r="99" ht="43.5" customHeight="1">
@@ -7158,8 +7161,8 @@
       </x:c>
       <x:c r="J99" s="5"/>
       <x:c r="K99" s="5"/>
-      <x:c r="L99" s="29" t="str">
-        <x:v>Ціна за запитом</x:v>
+      <x:c r="L99" s="29" t="n">
+        <x:v>1216.25</x:v>
       </x:c>
     </x:row>
     <x:row r="100" ht="43.5" customHeight="1">
@@ -7188,8 +7191,8 @@
       </x:c>
       <x:c r="J100" s="9"/>
       <x:c r="K100" s="9"/>
-      <x:c r="L100" s="29" t="str">
-        <x:v>Ціна за запитом</x:v>
+      <x:c r="L100" s="29" t="n">
+        <x:v>954.8</x:v>
       </x:c>
     </x:row>
     <x:row r="101" ht="43.5" customHeight="1">
@@ -7220,8 +7223,8 @@
         <x:v>60</x:v>
       </x:c>
       <x:c r="K101" s="5"/>
-      <x:c r="L101" s="29" t="str">
-        <x:v>Ціна за запитом</x:v>
+      <x:c r="L101" s="29" t="n">
+        <x:v>1588.4</x:v>
       </x:c>
     </x:row>
     <x:row r="102" ht="43.5" customHeight="1">
@@ -7250,8 +7253,8 @@
       </x:c>
       <x:c r="J102" s="9"/>
       <x:c r="K102" s="9"/>
-      <x:c r="L102" s="29" t="str">
-        <x:v>Ціна за запитом</x:v>
+      <x:c r="L102" s="29" t="n">
+        <x:v>258.69</x:v>
       </x:c>
     </x:row>
     <x:row r="103" ht="43.5" customHeight="1">
@@ -7365,7 +7368,7 @@
     <x:cfRule type="containsText" dxfId="8" priority="3" operator="containsText" text="очікується"/>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R191a28772fbb485a"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb3a57a8000eb4705"/>
 </x:worksheet>
 </file>
 
@@ -7414,7 +7417,8 @@
         <x:v>Статус</x:v>
       </x:c>
       <x:c r="G2" s="14" t="str">
-        <x:v>РРЦ, $ / од.</x:v>
+        <x:v>Ціна SunChe, $
+без ПДВ</x:v>
       </x:c>
     </x:row>
     <x:row r="3" ht="118.5" customHeight="1">
@@ -7438,7 +7442,7 @@
         <x:v>в наявності</x:v>
       </x:c>
       <x:c r="G3" s="18" t="n">
-        <x:v>1.56</x:v>
+        <x:v>1.38</x:v>
       </x:c>
     </x:row>
     <x:row r="4" ht="118.5" customHeight="1">
@@ -7462,7 +7466,7 @@
         <x:v>в наявності</x:v>
       </x:c>
       <x:c r="G4" s="18" t="n">
-        <x:v>1.08</x:v>
+        <x:v>0.99</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="118.5" customHeight="1">
@@ -7496,6 +7500,6 @@
     <x:cfRule type="containsText" dxfId="11" priority="3" operator="containsText" text="очікується"/>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc410bdf4a9254ea9"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R067812ef62114ac8"/>
 </x:worksheet>
 </file>
</xml_diff>